<commit_message>
Updated README and added requirements
</commit_message>
<xml_diff>
--- a/finance_report.xlsx
+++ b/finance_report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B2" t="n">
         <v>50000</v>
@@ -453,25 +453,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>27-06-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>60000</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Freelancing</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>27-06-2026</t>
+          <t>28-06-2026</t>
         </is>
       </c>
     </row>
@@ -486,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,73 +495,37 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>27-06-2026</t>
+          <t>28-06-2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B3" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Travel</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>27-06-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>27-06-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>27-06-2026</t>
+          <t>28-06-2026</t>
         </is>
       </c>
     </row>

</xml_diff>